<commit_message>
added import feature to personnel
</commit_message>
<xml_diff>
--- a/db/data/office_transactions.xlsx
+++ b/db/data/office_transactions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pradeep\Desktop\storemgmt\db\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E339535A-25A1-4EEA-B711-36A825809BB2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0179421-2A5C-4226-9626-3052B5C0988C}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20490" windowHeight="10920" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>